<commit_message>
King decision 14 Sep: park COMOBIL too (no WA/FB/trip this week); board refocused on OraCare + Sasse + NHICHS email; Tue batch becomes channel-qualified backfill
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -754,7 +754,7 @@
     <row r="6" ht="42" customHeight="1" s="25">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>COMOBIL / Groupe WAFO (Douala)</t>
+          <t>COMOBIL / Groupe WAFO (Douala) - PARKED 14 Sep (King decision)</t>
         </is>
       </c>
       <c r="B6" s="21" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>HOLD pending decision 14 Sep (no WA verified; no FB; email weak): (A) FB Page setup tonight sales/AMK-Facebook-Page-Setup.md -&gt; DM Wed; (B) Douala visit w/ QR. Concept hosted /comobil/.</t>
+          <t>#1 revival lead. Triggers: FB Page created -&gt; send pack §2 within 48h; Douala trip -&gt; walk-in w/ QR; comobil.com dark; WAFO referral. Concept hosted /comobil/.</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>review Fri</t>
         </is>
       </c>
     </row>
@@ -1165,10 +1165,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="25" min="1" max="1"/>
@@ -5739,6 +5739,41 @@
       <c r="K40" t="inlineStr">
         <is>
           <t>OraCare msg1 sent (video/file double-bind). King committed full demo folder incl canonical sjc-sasse-v2 + chapel photo + shots. AMK: oracare v3 (prices+assistant), comobil v1, sasse channel patch (form to email), hosting/previews bundle, week plan + pack + Pipeline-Status + W37 research.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>0 new sends EVE decision block</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>King phone-verified: COMOBIL + SAHISCOL not on WhatsApp; declined Facebook Page + Douala trip this week. Both parked with revival triggers (COMOBIL #1 revival). Kill list now OraCare + Sasse (+NHICHS email Tue). New sourcing rule: reachable channel before high score. Tue batch 8-10 channel-qualified D/E.</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6155,7 @@
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>PARKED 14 Sep (no WA; maintained template site; weak channel)</t>
+          <t>PARKED 14 Sep confirmed (no WA; maintained template site; weak channel)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -6219,12 +6254,12 @@
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>2 - HELD channel decision (no WA verified 14 Sep; no FB; email weak)</t>
+          <t>PARKED 14 Sep by King decision (channel, not pain: no WA/FB, weak email)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Decision 14 Sep: (A) AMK FB Page -&gt; DM Wed (sales/AMK-Facebook-Page-Setup.md); (B) Douala visit with QR. Concept hosted /comobil/.</t>
+          <t>#1 revival lead: triggers = AMK FB Page created (sales/AMK-Facebook-Page-Setup.md); Douala trip; comobil.com goes dark; WAFO referral. Concept hosted /comobil/, msg queued pack §2. Tue 22 deposit target withdrawn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tue 15 Buea walk-in batch: 10 routed stops, 7 new leads, printable WA QR cards, EN/FR gate scripts
- sales/Walk-In-Batch-2026-09-15.md: Molyko x3 (St Theresa, Salvation, St Bernard), Wokoko Summerset (1000 students), Bonduma x2 (NABESK, Baird), Great Soppo x3 (Baptist Comp, Inter caution, PCSS boarding), Muea stretch; timing, objections, contingent WA msgs for tonight's number checks
- sales/walkin/: QR PNGs (EN/FR deep links to AMK WA) + printable 9-card A4 sheet + builder (agency URL slot for later)
- CRM: new leads IDs 27-33 scored, enriched Salvation/PCSS/Frankfils/Marthlo; pipeline tab rows; Daily Ops rewritten for walk-in day
- sourcing channel logged: GCE Board accommodation-centre PDFs (verified active schools + quarters + candidate counts)
- Pipeline-Status + Weekly Plan updated; Sasse DM/email + NHICHS email slot around the route

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -689,7 +689,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="21.95" customHeight="1" s="25">
       <c r="A3" s="26" t="inlineStr">
         <is>
@@ -854,7 +853,6 @@
       </c>
       <c r="E10" s="21" t="n"/>
     </row>
-    <row r="11"/>
     <row r="12" ht="21.95" customHeight="1" s="25">
       <c r="A12" s="26" t="inlineStr">
         <is>
@@ -1165,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -1190,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA27"/>
+  <dimension ref="A1:AA34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="25" min="1" max="1"/>
@@ -3603,7 +3601,7 @@
       <c r="Z19" s="2" t="n"/>
       <c r="AA19" s="2" t="inlineStr">
         <is>
-          <t>4.1/5 (43 reviews, inovedu); tuition 213k–281k FCFA/yr. Presbyterian co-ed boarding. Quick verification could push to A.</t>
+          <t>4.1/5 (43 reviews, inovedu); tuition 213k–281k FCFA/yr. Presbyterian co-ed boarding. Quick verification could push to A. | Tue 15 walk-in Loop 2 (Great Soppo gate TBC); WA-check 652 075 229 + 675 533 321 Mon night; email pcss@yahoo.com; boarding hook + Presbyterian network angle; confessional principal-first.</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3726,7 @@
       <c r="Z20" s="2" t="n"/>
       <c r="AA20" s="2" t="inlineStr">
         <is>
-          <t>GCE centre 11402; 71% O-Level pass rate 2018 (concourscameroon). Verify before contact.</t>
+          <t>GCE centre 11402; 71% O-Level pass rate 2018 (concourscameroon). Verify before contact. | Tue 15 BACKUP walk-in if in quarter (Muea stretch swap).</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3851,7 @@
       <c r="Z21" s="2" t="n"/>
       <c r="AA21" s="2" t="inlineStr">
         <is>
-          <t>GCE centre 11412; accommodation centre for BHS Buea. Verify before contact.</t>
+          <t>GCE centre 11412; accommodation centre for BHS Buea. Verify before contact. | Tue 15 walk-in stop #2 Molyko; zero online contacts = gate visit solves it; capture principal WA + enrollment poster.</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3976,7 @@
       <c r="Z22" s="2" t="n"/>
       <c r="AA22" s="2" t="inlineStr">
         <is>
-          <t>GCE centre 22037 (technical streams). Verify before contact.</t>
+          <t>GCE centre 22037 (technical streams). Verify before contact. | Tue 15 BACKUP walk-in (technical streams angle).</t>
         </is>
       </c>
     </row>
@@ -4604,6 +4602,507 @@
       <c r="AA27" s="2" t="inlineStr">
         <is>
           <t>Confessional private secondary (ecolesaucameroun directory). Verify before contact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>St. Theresa International Bilingual Comprehensive College (STIBCCOL)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Buea (Molyko)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>EN/FR</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Page 100067292716772 (admissions-ongoing post Aug 2024)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>D/E - no site</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Yes (FB admissions posts)</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>via FB page (not listed)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>verify on walk-in</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Principal/proprietor (capture)</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>WALK-IN Tue 15 stop 1 + stibccol@yahoo.com</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Large GCE centre 11555 (~128 candidates 2024)</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>14</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Summerset Bilingual College (SMBICOL)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Buea (Wokoko)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>EN/FR</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>D/E - no site</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Likely (verify on gate)</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>not listed</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>verify on walk-in</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Proprietor/principal (capture)</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>WALK-IN Tue 15 stop 4 + smbicol@yahoo.com</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>~1,000 students / ~80 teachers (2021 paper); GCE centre 11447; founded 2000 lay private</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>15</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Walk-In-Batch-2026-09-15 FLAGSHIP stop: biggest enrollment of the day, zero web presence. Full 90s if allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Saint Bernard High School (SBHS)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Buea (Molyko)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>D/E - no site</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Yes - growth-stage</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>not listed</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>verify on walk-in</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Dr. Bernard Fomba (founder/proprietor, Oct 2020)</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>WALK-IN Tue 15 stop 3</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Forms 1-Upper 6th, general + commercial; ~247 at founding; GCE centre 12652</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
+        <v>12</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Walk-In-Batch-2026-09-15. Young school 2020 = hungry for growth, budget caution; founder decides alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NABESK Comprehensive College</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Buea (Bonduma)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>D/E - no site</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>not listed</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>verify on walk-in</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Principal (capture)</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>WALK-IN Tue 15 stop 5</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>GCE centre 11853; 83.5% O-level 2020; hosts 400+ external candidates = strong reputation</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>13</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Walk-In-Batch-2026-09-15. Hook: results buried in GCE PDFs, should be front page of own site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Baird Memorial College</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Buea (Bonduma)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>D/E - no site</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>not listed</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>verify on walk-in</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Principal (capture)</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>WALK-IN Tue 15 stop 6 (light, same road as NABESK)</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>GCE centre 11489; small (20-40 candidates)</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>7</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Walk-In-Batch-2026-09-15. Card + 2 min; deepen only if interest shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Baptist Comprehensive College</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Buea (Great Soppo)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Page lists +237 679 65 07 07</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>D/E - no site</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>+237 679 65 07 07</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>CHECK Mon night</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Principal; Baptist education office above</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>WA-CHECK then WALK-IN Tue 15 stop 7; bgccbuea@yahoo.com</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>GCE centre 11708</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>12</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Walk-In-Batch-2026-09-15. Confessional: principal first, ask 'who else decides?', offer forwardable version. Contingent WA msg in walk-in doc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>St. Sylvester International College</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Buea (Muea)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>EN/FR</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>D/E - no site</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>not listed</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>verify on walk-in</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Principal (capture)</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>WALK-IN Tue 15 STRETCH stop 10 (if ahead of schedule)</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>GCE centre 12908; 48 candidates 2025; international private</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>8</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Walk-In-Batch-2026-09-15. Swap for Frankfils/Marthlo depending on quarter. 'International' = fee capacity.</t>
         </is>
       </c>
     </row>
@@ -5788,7 +6287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="25" min="1" max="1"/>
@@ -6053,7 +6552,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15.75" customHeight="1" s="25">
       <c r="A8" s="16" t="inlineStr">
         <is>
@@ -6986,6 +7484,125 @@
       <c r="G36" t="inlineStr">
         <is>
           <t>1h reply; branch sheet + BANT in Outreach-Pack-2026-09-14 §1; host first (/oracare/), send concept-oracare-v3 (prices + assistant); FU1 Wed 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>St. Theresa International Bilingual Comprehensive College (STIBCCOL)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2 walk-in Tue 15</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Tue 15 walk-in (sales/Walk-In-Batch-2026-09-15.md): meet principal, get WA, book preview review; concept within 24h on warm yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Summerset Bilingual College (SMBICOL)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2 walk-in Tue 15</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Tue 15 walk-in (sales/Walk-In-Batch-2026-09-15.md): meet principal, get WA, book preview review; concept within 24h on warm yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Saint Bernard High School (SBHS)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2 walk-in Tue 15</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Tue 15 walk-in (sales/Walk-In-Batch-2026-09-15.md): meet principal, get WA, book preview review; concept within 24h on warm yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>NABESK Comprehensive College</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2 walk-in Tue 15</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Tue 15 walk-in (sales/Walk-In-Batch-2026-09-15.md): meet principal, get WA, book preview review; concept within 24h on warm yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Baird Memorial College</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2 walk-in Tue 15</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Tue 15 walk-in (sales/Walk-In-Batch-2026-09-15.md): meet principal, get WA, book preview review; concept within 24h on warm yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Baptist Comprehensive College</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2 walk-in Tue 15</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Tue 15 walk-in (sales/Walk-In-Batch-2026-09-15.md): meet principal, get WA, book preview review; concept within 24h on warm yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>St. Sylvester International College</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2 walk-in Tue 15</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Tue 15 walk-in (sales/Walk-In-Batch-2026-09-15.md): meet principal, get WA, book preview review; concept within 24h on warm yes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Invitation-first replan: digital Tue, async card-drop Wed, visits by invitation only
- sales/Invitation-First-Replan-2026-09-15.md: sure-WA table (Baptist 679, PCSS 652, Kinang 675 King-confirmed), pending-verify numbers (St Theresa 679 15 10 75 from official FB + active TikTok @stibccol; Baird 677s), two-step preview->invite-choice sequence, Wed sealed-envelope card-drop sweep for 5 numberless gates, exact Tue messages EN
- hosting/samples bundle (build_samples.py): public nameless templates to deploy as Vercel project for cold-preview links
- St Theresa: official number + active TikTok recorded; Summerset FB dead since 2015, no phone online -> email + named envelope card drop
- CRM channels rewritten for all 10; Daily Ops rebuilt as Tue digital-first / Wed sweep / invited visits Wed PM-Fri; old route doc banner-superseded; deep dives patched

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Tue 08:30 WhatsApp 652 075 229 (CONFIRMED on WA; official line); Kinang 675 533 321 door-opener at noon if silent; visit by invitation</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Wed 16 async card-drop sweep (Salvation Molyko near CUIB); no meeting, sealed envelope to principal; visit only by invitation</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -4646,12 +4646,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>via FB page (not listed)</t>
+          <t>+237 679 15 10 75 (official FB page intro; King to WA-verify); secondary 677 36 19 11 low confidence</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>verify on walk-in</t>
+          <t>CHECK 679 15 10 75 tonight</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>WALK-IN Tue 15 stop 1 + stibccol@yahoo.com</t>
+          <t>Tue 15: TikTok DM @stibccol (active to 14 Sep 2026) + WhatsApp 679 15 10 75 if confirmed</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm.</t>
+          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch.</t>
         </is>
       </c>
     </row>
@@ -4702,6 +4702,11 @@
           <t>EN/FR</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Page facebook.com/summerset.bilingual.college INACTIVE since Dec 2015 (stray email dadariodelanuez@yahoo.com - do not use)</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>None found</t>
@@ -4719,12 +4724,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>not listed</t>
+          <t>not published anywhere</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>verify on walk-in</t>
+          <t>none found</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -4734,7 +4739,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>WALK-IN Tue 15 stop 4 + smbicol@yahoo.com</t>
+          <t>Tue parallel email smbicol@yahoo.com (weak); Wed async card-drop addressed to Principal Tata; invited visit only after</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -4752,7 +4757,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15 FLAGSHIP stop: biggest enrollment of the day, zero web presence. Full 90s if allowed. | DEEP DIVE 14 Sep: LOCATION Check Point (Wokoko), opposite ENAMEN Pharmacy. Principal Mr Yerima Samson Tata (Cameroon Tribune Jun/Sep 2026). LIVE PAIN: principal publicly reported slower 2026/27 enrollment (parents arriving Oct) while spending on repainting/benches. Facilities: science lab, computer lab + internet, band, generator, reservoir; UNIQUE evening school 15:30. Mission text commits to technology + bilingualism. ~1,350 GCE candidates hosted 2026.</t>
+          <t>Walk-In-Batch-2026-09-15 FLAGSHIP stop: biggest enrollment of the day, zero web presence. Full 90s if allowed. | DEEP DIVE 14 Sep: LOCATION Check Point (Wokoko), opposite ENAMEN Pharmacy. Principal Mr Yerima Samson Tata (Cameroon Tribune Jun/Sep 2026). LIVE PAIN: principal publicly reported slower 2026/27 enrollment (parents arriving Oct) while spending on repainting/benches. Facilities: science lab, computer lab + internet, band, generator, reservoir; UNIQUE evening school 15:30. Mission text commits to technology + bilingualism. ~1,350 GCE candidates hosted 2026. | INVITATION-FIRST 14 Sep: NO reachable digital channel - no phone online, FB dead since 2015. Plan: email Tue + sealed-envelope card drop Wed (hand-addressed to Principal Yerima Samson Tata, opposite ENAMEN Pharmacy); QR inbound = they initiate; visit by invitation only.</t>
         </is>
       </c>
     </row>
@@ -4807,7 +4812,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>WALK-IN Tue 15 stop 3</t>
+          <t>Wed 16 async card-drop sweep (SBHS Garden Park opposite Orange, attn Dr Fomba); no meeting, sealed envelope to principal; visit only by invitation</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -4875,7 +4880,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>WALK-IN Tue 15 stop 5</t>
+          <t>Wed 16 async card-drop sweep (NABESK Nabesk junction); no meeting, sealed envelope to principal; visit only by invitation</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4961,7 +4966,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate.</t>
+          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate. | INVITATION-FIRST 14 Sep: WA-check 677 87 53 95 + 677 78 04 05 profile attribution tonight; message only if site dead AND number on WA (text in replan section 4); otherwise Wed card drop same road as NABESK.</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5021,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>WA-CHECK then WALK-IN Tue 15 stop 7; bgccbuea@yahoo.com</t>
+          <t>Tue 08:30 WhatsApp 679 65 07 07 (CONFIRMED on WA King 14 Sep; school line) then preview link; invite-choice walkthrough Thu/Fri; gate visit only if invited</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -5084,7 +5089,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>WALK-IN Tue 15 STRETCH stop 10 (if ahead of schedule)</t>
+          <t>Wed 16 async card-drop sweep (St Sylvester Muea (fold in only if Muea trip)); no meeting, sealed envelope to principal; visit only by invitation</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -5162,7 +5167,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>WALK-IN Tue 15 stop 8 (replaces disqualified Inter Comp)</t>
+          <t>Hold for diocesan motion behind Sasse; fold card/visit into Great Soppo/Bokwaongo invited trip; do not cold-gate</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">

</xml_diff>

<commit_message>
Solidarity: 677 61 57 57 not on WhatsApp (King-checked); MITOC leads Tuesday 08:35
- Clinic line demoted to voice-only; never cold-called
- Remaining WA candidate: SHF-CIG admin 677 61 12 07 (check profile answers as clinic); fallback Wed sealed envelope to 'current medical director or clinic manager'
- CRM 36 channel/phone/notes/follow-up (Wed 16 Sep) updated; Daily Ops rebuilt (59 rows); dossier/replan/pipeline log updated; MITOC msg 1 confirmed ready

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -5308,12 +5308,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>CLINIC LINE 677 61 57 57 (ORG-LIKELY: GBP+elidge+medicoor; King WA-profile check tonight); landline 2 33 32 31 31; admin candidate 677 61 12 07 (UN NGO registry, unverified)</t>
+          <t>CLINIC LINE 677 61 57 57 (ORG-LIKELY: GBP+elidge+medicoor) BUT NOT ON WHATSAPP (King 15 Sep, voice only); landline 2 33 32 31 31; admin WA candidate 677 61 12 07 (UN NGO registry, unverified); 691 63 29 41 = Dr Njang personal, HOLD</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>VERIFY 677 61 57 57 as clinic line tonight. DO NOT TEXT 691 63 29 41 about Solidarity: King confirms it is Dr Njang's PERSONAL WhatsApp; his current role at the clinic is unconfirmed and he co-owns a competing lab</t>
+          <t>677 61 57 57 NOT on WhatsApp (King 15 Sep); fallback admin 677 61 12 07 unverified; 691 63 29 41 = Dr Njang personal, HOLD</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -5323,7 +5323,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Tue 15 Sep 08:35 WhatsApp msg 1 (Clinic-Batch section 1, NO personal names) to clinic line 677 61 57 57 after King's WA-profile check; asks for current medical director OR clinic manager. Yes = nameless /sample-clinic.html + invite choice; named within 24h</t>
+          <t>WA blocked on clinic line -&gt; check SHF-CIG admin 677 61 12 07; else Wed 16 Sep sealed envelope to 'current medical director or clinic manager'</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -5356,12 +5356,12 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>Tue 15 Sep</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>Clinic lead #1, research-standard corrected 15 Sep (see sales/RESEARCH-STANDARD.md error #1). Not-for-profit CIG founded Aug 1998 by late Dr Peter Nde Fon (UB public health chair, obituary verified). GBP 4.0 stars/54 reviews/21 photos/24h, Untarred Malingo St plus code 575J+7M, NO website ('Add website'), medicoor unclaimed+stale (still lists deceased founder), X @SolidarityHeal1 since May 2021. Services: gen med, vaccination, surgery, lab panels, maternity, ultrasound/X-ray; reviews cite cardiologist+pharmacy; Zenithe accredited. Among Buea district top-3 most-solicited facilities (PAMJ 2023, BMRI 2025). Pitch: attach bilingual site+WA booking+same-day lab results to GBP; foundation/grant visibility; claim medicoor; 24h emergency bar. FUs M+2/M+4/M+7.</t>
+          <t>Clinic lead #1, research-standard corrected 15 Sep (see sales/RESEARCH-STANDARD.md error #1). Not-for-profit CIG founded Aug 1998 by late Dr Peter Nde Fon (UB public health chair, obituary verified). GBP 4.0 stars/54 reviews/21 photos/24h, Untarred Malingo St plus code 575J+7M, NO website ('Add website'), medicoor unclaimed+stale (still lists deceased founder), X @SolidarityHeal1 since May 2021. Services: gen med, vaccination, surgery, lab panels, maternity, ultrasound/X-ray; reviews cite cardiologist+pharmacy; Zenithe accredited. Among Buea district top-3 most-solicited facilities (PAMJ 2023, BMRI 2025). Pitch: attach bilingual site+WA booking+same-day lab results to GBP; foundation/grant visibility; claim medicoor; 24h emergency bar. FUs M+2/M+4/M+7. [15 Sep send morning: 677 61 57 57 not registered on WhatsApp per King; voice line only, never cold-call; MITOC now leads Tue 08:35; Solidarity -&gt; admin-line check, else Wed sealed card]</t>
         </is>
       </c>
     </row>
@@ -5570,10 +5570,6 @@
           <t>not contacted</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
       <c r="Z39" t="inlineStr">
         <is>
           <t>research then schedule</t>

</xml_diff>

<commit_message>
MITOC: WA Business profile verified (catalogue, 09-18h, accessories + computer/swimming glasses); site v2 + final msg 1
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>KING TO VERIFY 678 90 89 62 on WA (number from official FB intro)</t>
+          <t>678 90 89 62 = ORG-CONFIRMED WA Business account 'MITOC' (King 15 Sep); catalogue live; bio: examine/prescribe/fit lenses + lens accessories + computer &amp; swimming glasses; hours 09:00-18:00</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Tue 15 Sep 08:35 WhatsApp msg 1 (Clinic-Batch §2, KING PRIORITY) -&gt; yes = nameless /sample-clinic.html (optic re-skin promised in 24h) + invite choice</t>
+          <t>WhatsApp Business (org account) - msg 1 ready; named preview https://mitoc-concept.vercel.app after warm yes</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>Clinic lead #2. Pitch hooks: invisible on Google (FB-only), eye-test booking on WA, frames + FCFA lens prices bilingual, student catchment Molyko. Smaller scope than Solidarity - quote by scope, never discount. Follow-ups M+2/M+4/M+7. [15 Sep: named concept ready /mitoc.html, cobalt+cream, 140 EN/FR pairs, demo WA routing AMK; send only after warm yes + 678 90 89 62 WA-profile check]</t>
+          <t>Clinic lead #2. Pitch hooks: invisible on Google (FB-only), eye-test booking on WA, frames + FCFA lens prices bilingual, student catchment Molyko. Smaller scope than Solidarity - quote by scope, never discount. Follow-ups M+2/M+4/M+7. [15 Sep: named concept ready /mitoc.html, cobalt+cream, 140 EN/FR pairs, demo WA routing AMK; send only after warm yes + 678 90 89 62 WA-profile check] [15 Sep 11:39 KING-VERIFIED business profile; email ateasomcollins@gmail.com (unused); site updated w/ hours + computer/swimming/accessories, 144 EN/FR pairs]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
School pair: final Baptist/PCSS msg 1 (preview-ready leverage, network proof for PCSS); log MITOC sent
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -5459,12 +5459,12 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>scheduled Tue</t>
+          <t>YES 15 Sep ~11:45 WA msg 1 (catalogue-ack variant); awaiting reply</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>Tue 15 Sep</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">

</xml_diff>

<commit_message>
PCSS: 652 075 229 verified as org WA Business operated by Namondo Elangwe (likely principal); named msg variant; Kinang fallback moved to M+2
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -3536,12 +3536,12 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>N/V</t>
+          <t>652 075 229 = ORG WA Business 'PCSS BUEA', contact person Namondo Elangwe (King screenshot 15 Sep); same woman = 'Madam Namondo Alexander', school's own GPEN network contact since 2021 -&gt; LIKELY principal/senior proprietor (title UNVERIFIED, do not state)</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Headmaster (N/V); staff contact: Kinang Edwin Ngenge, 675 533 321</t>
+          <t>Namondo Elangwe ('Madam Namondo') - LIKELY principal, VERIFIED name only; title confirm at gate</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -3601,7 +3601,7 @@
       <c r="Z19" s="2" t="n"/>
       <c r="AA19" s="2" t="inlineStr">
         <is>
-          <t>4.1/5 (43 reviews, inovedu); tuition 213k–281k FCFA/yr. Presbyterian co-ed boarding. Quick verification could push to A. | Tue 15 walk-in Loop 2 (Great Soppo gate TBC); WA-check 652 075 229 + 675 533 321 Mon night; email pcss@yahoo.com; boarding hook + Presbyterian network angle; confessional principal-first. | DEEP DIVE 14 Sep: 652 075 229 = official line self-listed on GPENreformation (confirmed on WA King 14 Sep = school line, not principal personal). 675 533 321 = Kinang Edwin Ngenge, staff/language teacher &amp; network partnership contact (NOT decision-maker; internal champion). Sister school PCSS Bonamoussadi Douala already runs pcssbonamoussadi.online with WhatsApp = network precedent (do not name). Boarding 700+ = headline hook.</t>
+          <t>4.1/5 (43 reviews, inovedu); tuition 213k–281k FCFA/yr. Presbyterian co-ed boarding. Quick verification could push to A. | Tue 15 walk-in Loop 2 (Great Soppo gate TBC); WA-check 652 075 229 + 675 533 321 Mon night; email pcss@yahoo.com; boarding hook + Presbyterian network angle; confessional principal-first. | DEEP DIVE 14 Sep: 652 075 229 = official line self-listed on GPENreformation (confirmed on WA King 14 Sep = school line, not principal personal). 675 533 321 = Kinang Edwin Ngenge, staff/language teacher &amp; network partnership contact (NOT decision-maker; internal champion). Sister school PCSS Bonamoussadi Douala already runs pcssbonamoussadi.online with WhatsApp = network precedent (do not name). Boarding 700+ = headline hook. [15 Sep: business profile verified; msg 1 addressed 'Madam Namondo', direct-ask variant; Kinang fallback moved to M+2, not same day]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Baptist msg 1 sent (M+2 = 17 Sep)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -5037,6 +5037,16 @@
           <t>B+</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>YES 15 Sep ~12:00 WA msg 1 (preview-ready variant); one tick as of send, awaiting</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="AA33" t="inlineStr">
         <is>
           <t>Walk-In-Batch-2026-09-15. Confessional: principal first, ask 'who else decides?', offer forwardable version. Contingent WA msg in walk-in doc. | DEEP DIVE 14 Sep: 679 65 07 07 confirmed on WA (King) — attribution = number published on the college FB page intro (official school line, role unknown; likely admin/proprietor; verify profile photo/name tonight). Baptist confessional -&gt; principal then Baptist education office; ask who else decides. bgccbuea@yahoo.com.</t>

</xml_diff>

<commit_message>
Reclassify missionary/confessional secondaries as BOARD-BUYERs (King): park PCSS before send, Baptist inbound-only, network-website claim corrected (error log #2)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -2226,7 +2226,7 @@
       <c r="Z8" s="2" t="n"/>
       <c r="AA8" s="2" t="inlineStr">
         <is>
-          <t>Active FB page (1,785 likes, school fundraiser). Need phone before outreach — try FB message first.</t>
+          <t>Active FB page (1,785 likes, school fundraiser). Need phone before outreach — try FB message first. [BOARD-BUYER 15 Sep King: Presbyterian/congregation school; principal cannot sign; park from 30-day push; network-level play later]</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       <c r="Z15" s="2" t="n"/>
       <c r="AA15" s="2" t="inlineStr">
         <is>
-          <t>Respected Christian boarding school, consistent GCE results (237zoom ranking #8). No website found. Verify FB activity before outreach.</t>
+          <t>Respected Christian boarding school, consistent GCE results (237zoom ranking #8). No website found. Verify FB activity before outreach. [BOARD-BUYER 15 Sep King: Baptist mission school; centralized Baptist education office; park, inbound only]</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       <c r="Z18" s="2" t="n"/>
       <c r="AA18" s="2" t="inlineStr">
         <is>
-          <t>THE #1 DEMO TARGET. 100% exam success tradition; SOBA alumni network (FCFA 23M scholarships 2025); Catholic all-boys; sajoscol@gmail.com. No website = missing destination for their active attention. DEMO BUILT: sjc-sasse-homepage.html. 2012 'Best School in West Africa' + 2013 'Best School in Cameroon' (Fondation Terre d'accueil) — demo material. WhatsApp 677 195 500 NOT available (King 09/09) → TIKTOK DM @SJC - The Republic + email sajoscol@gmail.com + call. Diocesan education line: +237 334 745 678. | Canonical concept demos/sjc-sasse-v2.html (King file committed 14 Sep, 123 pairs, chapel photo; AMK patched form to email sajoscol@gmail.com since 677 195 500 is not on WhatsApp; landline/email/TikTok links added).</t>
+          <t>THE #1 DEMO TARGET. 100% exam success tradition; SOBA alumni network (FCFA 23M scholarships 2025); Catholic all-boys; sajoscol@gmail.com. No website = missing destination for their active attention. DEMO BUILT: sjc-sasse-homepage.html. 2012 'Best School in West Africa' + 2013 'Best School in Cameroon' (Fondation Terre d'accueil) — demo material. WhatsApp 677 195 500 NOT available (King 09/09) → TIKTOK DM @SJC - The Republic + email sajoscol@gmail.com + call. Diocesan education line: +237 334 745 678. | Canonical concept demos/sjc-sasse-v2.html (King file committed 14 Sep, 123 pairs, chapel photo; AMK patched form to email sajoscol@gmail.com since 677 195 500 is not on WhatsApp; landline/email/TikTok links added). [BOARD-BUYER 15 Sep King: Catholic diocesan college; bishop/education office decide; TikTok 15 Sep treated as inbound-only seed, no FU chase]</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO - parked pre-send 15 Sep (BOARD-BUYER)</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
@@ -3601,7 +3601,7 @@
       <c r="Z19" s="2" t="n"/>
       <c r="AA19" s="2" t="inlineStr">
         <is>
-          <t>4.1/5 (43 reviews, inovedu); tuition 213k–281k FCFA/yr. Presbyterian co-ed boarding. Quick verification could push to A. | Tue 15 walk-in Loop 2 (Great Soppo gate TBC); WA-check 652 075 229 + 675 533 321 Mon night; email pcss@yahoo.com; boarding hook + Presbyterian network angle; confessional principal-first. | DEEP DIVE 14 Sep: 652 075 229 = official line self-listed on GPENreformation (confirmed on WA King 14 Sep = school line, not principal personal). 675 533 321 = Kinang Edwin Ngenge, staff/language teacher &amp; network partnership contact (NOT decision-maker; internal champion). Sister school PCSS Bonamoussadi Douala already runs pcssbonamoussadi.online with WhatsApp = network precedent (do not name). Boarding 700+ = headline hook. [15 Sep: business profile verified; msg 1 addressed 'Madam Namondo', direct-ask variant; Kinang fallback moved to M+2, not same day]</t>
+          <t>4.1/5 (43 reviews, inovedu); tuition 213k–281k FCFA/yr. Presbyterian co-ed boarding. Quick verification could push to A. | Tue 15 walk-in Loop 2 (Great Soppo gate TBC); WA-check 652 075 229 + 675 533 321 Mon night; email pcss@yahoo.com; boarding hook + Presbyterian network angle; confessional principal-first. | DEEP DIVE 14 Sep: 652 075 229 = official line self-listed on GPENreformation (confirmed on WA King 14 Sep = school line, not principal personal). 675 533 321 = Kinang Edwin Ngenge, staff/language teacher &amp; network partnership contact (NOT decision-maker; internal champion). Sister school PCSS Bonamoussadi Douala already runs pcssbonamoussadi.online with WhatsApp = network precedent (do not name). Boarding 700+ = headline hook. [15 Sep: business profile verified; msg 1 addressed 'Madam Namondo', direct-ask variant; Kinang fallback moved to M+2, not same day] [BOARD-BUYER 15 Sep King: PCC college; PARKED before send, no msg 1, no Kinang text; network deliberately website-free; future PCC education-secretary proposal]</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       <c r="Z21" s="2" t="n"/>
       <c r="AA21" s="2" t="inlineStr">
         <is>
-          <t>GCE centre 11412; accommodation centre for BHS Buea. Verify before contact. | Tue 15 walk-in stop #2 Molyko; zero online contacts = gate visit solves it; capture principal WA + enrollment poster. | DEEP DIVE 14 Sep: located near Baptist church (Ndongo) and CUIB, Molyko; technical A-Level 91.7% pass 2016 incl Accounting; GCE centres 11412 + 22089, hosts external candidates. Zero online contacts = walk-in only; confirm faith affiliation + enrollment at gate.</t>
+          <t>GCE centre 11412; accommodation centre for BHS Buea. Verify before contact. | Tue 15 walk-in stop #2 Molyko; zero online contacts = gate visit solves it; capture principal WA + enrollment poster. | DEEP DIVE 14 Sep: located near Baptist church (Ndongo) and CUIB, Molyko; technical A-Level 91.7% pass 2016 incl Accounting; GCE centres 11412 + 22089, hosts external candidates. Zero online contacts = walk-in only; confirm faith affiliation + enrollment at gate. [VERIFY GOVERNANCE at gate: possibly faith-founded; confirm OWNER-BUYER proprietor vs BOARD-BUYER before any pitch]</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       <c r="Z27" s="2" t="n"/>
       <c r="AA27" s="2" t="inlineStr">
         <is>
-          <t>Confessional private secondary (ecolesaucameroun directory). Verify before contact.</t>
+          <t>Confessional private secondary (ecolesaucameroun directory). Verify before contact. [BOARD-BUYER 15 Sep: Presbyterian Girls Limbe; park per missionary reclassification; verify only if inbound]</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch.</t>
+          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan]</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15 FLAGSHIP stop: biggest enrollment of the day, zero web presence. Full 90s if allowed. | DEEP DIVE 14 Sep: LOCATION Check Point (Wokoko), opposite ENAMEN Pharmacy. Principal Mr Yerima Samson Tata (Cameroon Tribune Jun/Sep 2026). LIVE PAIN: principal publicly reported slower 2026/27 enrollment (parents arriving Oct) while spending on repainting/benches. Facilities: science lab, computer lab + internet, band, generator, reservoir; UNIQUE evening school 15:30. Mission text commits to technology + bilingualism. ~1,350 GCE candidates hosted 2026. | INVITATION-FIRST 14 Sep: NO reachable digital channel - no phone online, FB dead since 2015. Plan: email Tue + sealed-envelope card drop Wed (hand-addressed to Principal Yerima Samson Tata, opposite ENAMEN Pharmacy); QR inbound = they initiate; visit by invitation only.</t>
+          <t>Walk-In-Batch-2026-09-15 FLAGSHIP stop: biggest enrollment of the day, zero web presence. Full 90s if allowed. | DEEP DIVE 14 Sep: LOCATION Check Point (Wokoko), opposite ENAMEN Pharmacy. Principal Mr Yerima Samson Tata (Cameroon Tribune Jun/Sep 2026). LIVE PAIN: principal publicly reported slower 2026/27 enrollment (parents arriving Oct) while spending on repainting/benches. Facilities: science lab, computer lab + internet, band, generator, reservoir; UNIQUE evening school 15:30. Mission text commits to technology + bilingualism. ~1,350 GCE candidates hosted 2026. | INVITATION-FIRST 14 Sep: NO reachable digital channel - no phone online, FB dead since 2015. Plan: email Tue + sealed-envelope card drop Wed (hand-addressed to Principal Yerima Samson Tata, opposite ENAMEN Pharmacy); QR inbound = they initiate; visit by invitation only. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan]</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Young school 2020 = hungry for growth, budget caution; founder decides alone. | DEEP DIVE 14 Sep: located former HIMS Campus, Garden Park Molyko, opposite Orange Cameroon; motto Knowledge-Fidelity-Integrity; founder/proprietor Dr Bernard Fomba (ask by name, decides alone); 134 candidates at one 2025 session.</t>
+          <t>Walk-In-Batch-2026-09-15. Young school 2020 = hungry for growth, budget caution; founder decides alone. | DEEP DIVE 14 Sep: located former HIMS Campus, Garden Park Molyko, opposite Orange Cameroon; motto Knowledge-Fidelity-Integrity; founder/proprietor Dr Bernard Fomba (ask by name, decides alone); 134 candidates at one 2025 session. [VERIFY GOVERNANCE at gate: saint name but young 2020 founder-led? confirm lay proprietor decides before pitching]</t>
         </is>
       </c>
     </row>
@@ -4898,7 +4898,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Hook: results buried in GCE PDFs, should be front page of own site. | DEEP DIVE 14 Sep: school gives its name to Nabesk junction, Bonduma (press landmark Mar 2025); 83.5% O-level 2020; external candidate host (214/187/401 in 2025 movement lists). Ask who founded it (name may derive from proprietor).</t>
+          <t>Walk-In-Batch-2026-09-15. Hook: results buried in GCE PDFs, should be front page of own site. | DEEP DIVE 14 Sep: school gives its name to Nabesk junction, Bonduma (press landmark Mar 2025); 83.5% O-level 2020; external candidate host (214/187/401 in 2025 movement lists). Ask who founded it (name may derive from proprietor). [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan]</t>
         </is>
       </c>
     </row>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate. | INVITATION-FIRST 14 Sep: WA-check 677 87 53 95 + 677 78 04 05 profile attribution tonight; message only if site dead AND number on WA (text in replan section 4); otherwise Wed card drop same road as NABESK.</t>
+          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate. | INVITATION-FIRST 14 Sep: WA-check 677 87 53 95 + 677 78 04 05 profile attribution tonight; message only if site dead AND number on WA (text in replan section 4); otherwise Wed card drop same road as NABESK. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan]</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Confessional: principal first, ask 'who else decides?', offer forwardable version. Contingent WA msg in walk-in doc. | DEEP DIVE 14 Sep: 679 65 07 07 confirmed on WA (King) — attribution = number published on the college FB page intro (official school line, role unknown; likely admin/proprietor; verify profile photo/name tonight). Baptist confessional -&gt; principal then Baptist education office; ask who else decides. bgccbuea@yahoo.com.</t>
+          <t>Walk-In-Batch-2026-09-15. Confessional: principal first, ask 'who else decides?', offer forwardable version. Contingent WA msg in walk-in doc. | DEEP DIVE 14 Sep: 679 65 07 07 confirmed on WA (King) — attribution = number published on the college FB page intro (official school line, role unknown; likely admin/proprietor; verify profile photo/name tonight). Baptist confessional -&gt; principal then Baptist education office; ask who else decides. bgccbuea@yahoo.com. [BOARD-BUYER 15 Sep King: Baptist Comp.; msg 1 SENT 15 Sep (one tick) -&gt; inbound only, NO FU chase, NO cold walk-in; route via Baptist education office if reply asks for HQ]</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Swap for Frankfils/Marthlo depending on quarter. 'International' = fee capacity.</t>
+          <t>Walk-In-Batch-2026-09-15. Swap for Frankfils/Marthlo depending on quarter. 'International' = fee capacity. [VERIFY GOVERNANCE at gate: 'international' may be lay; confirm not diocesan before investing]</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Catholic diocesan pipeline (same motion as Sasse): principal first, offer forwardable preview, ask when Education Secretariat next meets; multi-college upside. Bokwaongo uphill past Great Soppo. Source: bueadiocese.org 18 Feb 2026.</t>
+          <t>Walk-In-Batch-2026-09-15. Catholic diocesan pipeline (same motion as Sasse): principal first, offer forwardable preview, ask when Education Secretariat next meets; multi-college upside. Bokwaongo uphill past Great Soppo. Source: bueadiocese.org 18 Feb 2026. [BOARD-BUYER: Catholic diocesan; hold per Sasse motion; never cold-drop]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Baird GO ops: CRM/Daily-Ops refresh, deterministic deploy zip + site/DEPLOY runbook
- leads: patch_baird_go.py applied (27 SENT 1-tick image-on-reply, 31 GO with
  personal-line/proprietress notes, 37 MITOC FU1 17/FU2 19/FU3 22); Daily Ops
  rebuilt with mockup rule, deploy gate, Solidarity image-first WA leg
- hosting/build_site_zip.py: deterministic 13-file amk-site.zip (local smoke
  test all-200, internal links resolve); site/DEPLOY.md runbook for amk-cm
- replan/status logs: DNS-dead recheck, Google-index correction, 13-file bundle

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Tue 15 Sep 15:45 WhatsApp msg 1 (replan §4); TikTok @stibccol DM Wed only if WA silent (no same-morning double touch)</t>
+          <t>SENT by King ~15:45 Tue 15 Sep (one grey tick; text-only). No chase; TikTok @stibccol DM = Wed second touch only if WA stays silent. On warm reply: attach demos/shots/mockup-secondary-wa.jpg + live /sample-secondary.html link, then Thu/Fri walkthrough choice</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan]</t>
+          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM: msg 1 out (1 tick, not yet delivered to handset). Personal WA line (lay private = likely proprietor pocket = buyer). Mockup image went to later schools first; include image with the link on reply.</t>
         </is>
       </c>
     </row>
@@ -4928,7 +4928,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>bairdmemorial.com DEAD - confirmed on King's phone 14 Sep (full pitch, not refresh)</t>
+          <t>bairdmemorial.com DNS-DEAD re-verified 15 Sep 13:35 (apex+www NXDOMAIN; Google still indexes the dead Home + /about-us -&gt; say 'leads parents nowhere', never 'finds nothing')</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Tue 15 Sep 16:00 WhatsApp msg 1 FULL pitch (replan §4); if silent, sealed card in Wed Limbe sweep; invited Bonduma visit only after</t>
+          <t>GO (King 'proceed' 15 Sep PM): attach demos/shots/mockup-secondary-wa.jpg FIRST, then recipient-neutral msg (replan §4) to WA 677 87 53 95; pre-tap open bairdmemorial.com once, swap para 3 if it loads; Wed sealed card in Limbe sweep if silent; invited visit only</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate. | INVITATION-FIRST 14 Sep: WA-check 677 87 53 95 + 677 78 04 05 profile attribution tonight; message only if site dead AND number on WA (text in replan section 4); otherwise Wed card drop same road as NABESK. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan]</t>
+          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate. | INVITATION-FIRST 14 Sep: WA-check 677 87 53 95 + 677 78 04 05 profile attribution tonight; message only if site dead AND number on WA (text in replan section 4); otherwise Wed card drop same road as NABESK. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM GO: 95 line is a PERSONAL WA account (man's profile photo, no business profile); their OWN old dead site names PROPRIETRESS Madam Mary Forju (also Mr Ndichafah Fredrick, extra nums 652 24 80 21/677 16 98 66/673 40 40 69, gmail/outlook/yahoo boxes - record only, never open). Holder of 95 unknown (principal/bursar/family possible) -&gt; msg asks 'proprietor or the principal?', never names her, never references the photo. Never mock old copy; ask who built it/last touched on warm reply.</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>WhatsApp Business (org account) - msg 1 ready; named preview https://mitoc-concept.vercel.app after warm yes</t>
+          <t>SENT msg 1 Tue (two ticks, awaiting reply). No chase same day; FU1 Thu 17 / FU2 Sat 19 / FU3 Tue 22 Sep (OWNER-BUYER only, then stop). Warm yes -&gt; https://mitoc-concept.vercel.app + 10-min shop visit vs all-on-WhatsApp; amk-cm /mitoc.html stays 404 until King redeploys amk-site.zip</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">

</xml_diff>

<commit_message>
Clinic concept renamed Bonabéri Medical Centre (Douala); Baird msg 1 SENT 14:41
- build_sample_clinic.py emits clinic-bonaberi.html fully renamed (brand x10,
  Douala eyebrow/address, BMC booking refs, canonical+history URLs); 150/150
  pairs and AMK demo WA routing intact; sample-clinic.html removed (404 correct)
- index links (x2), sitemap, zip builder, hosting mirror repointed; clinic
  thumbnail + mockup-clinic (+wa.jpg) regenerated with Douala branding
- King's live upload was a partial hand-rename (Buea eyebrow/Molyko leftovers);
  canonical redeploy via amk-site.zip completes it; DEPLOY.md + replan updated
- Baird 31 marked SENT 14:41 (image+text, one tick); sent text used the
  first-draft 'find nothing at all' line -> soft-ack reply branch documented
- CRM 36 rename notes; Daily Ops rebuilt; bundle smoke-tested (new 200/old 404)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -4964,9 +4964,14 @@
           <t>B+</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>YES 15 Sep 14:41 WA (mockup image + msg 1; one tick)</t>
+        </is>
+      </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate. | INVITATION-FIRST 14 Sep: WA-check 677 87 53 95 + 677 78 04 05 profile attribution tonight; message only if site dead AND number on WA (text in replan section 4); otherwise Wed card drop same road as NABESK. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM GO: 95 line is a PERSONAL WA account (man's profile photo, no business profile); their OWN old dead site names PROPRIETRESS Madam Mary Forju (also Mr Ndichafah Fredrick, extra nums 652 24 80 21/677 16 98 66/673 40 40 69, gmail/outlook/yahoo boxes - record only, never open). Holder of 95 unknown (principal/bursar/family possible) -&gt; msg asks 'proprietor or the principal?', never names her, never references the photo. Never mock old copy; ask who built it/last touched on warm reply.</t>
+          <t>Walk-In-Batch-2026-09-15 stop 6 light. Boarding 'inclusive' high school behind public tap Bonduma; bairdmemorial@yahoo.com; GCE 11489 (small); active CSDC inter-school events 2025. | DEEP DIVE 14 Sep: ALREADY HAS self-built website bairdmemorial.com (visible typos 'bording/Accademic', did not open externally). Phone-check tonight: DEAD = full D pitch ('I tried opening it before coming'); WORKS = card + soft refresh/upsell line, never criticise at gate. | INVITATION-FIRST 14 Sep: WA-check 677 87 53 95 + 677 78 04 05 profile attribution tonight; message only if site dead AND number on WA (text in replan section 4); otherwise Wed card drop same road as NABESK. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM GO: 95 line is a PERSONAL WA account (man's profile photo, no business profile); their OWN old dead site names PROPRIETRESS Madam Mary Forju (also Mr Ndichafah Fredrick, extra nums 652 24 80 21/677 16 98 66/673 40 40 69, gmail/outlook/yahoo boxes - record only, never open). Holder of 95 unknown (principal/bursar/family possible) -&gt; msg asks 'proprietor or the principal?', never names her, never references the photo. Never mock old copy; ask who built it/last touched on warm reply. | SENT 14:41 by King, single tick (delivered-pending). Next: 1h watch to 21:00; warm reply -&gt; live /sample-secondary.html + caption + Thu/Fri choice; silence -&gt; Wed sealed gate card in Limbe sweep; FUs M+2/M+4/M+7 OWNER-BUYER only after Wed card.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5361,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>nameless sample-clinic.html concept built 15 Sep (Forest palette)</t>
+          <t>nameless clinic-bonaberi.html (Bonabéri Medical Centre, Douala; Forest palette; was Molyko Medical Centre/sample-clinic.html, renamed by King 15 Sep PM)</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -5371,7 +5376,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>Clinic lead #1, research-standard corrected 15 Sep (see sales/RESEARCH-STANDARD.md error #1). Not-for-profit CIG founded Aug 1998 by late Dr Peter Nde Fon (UB public health chair, obituary verified). GBP 4.0 stars/54 reviews/21 photos/24h, Untarred Malingo St plus code 575J+7M, NO website ('Add website'), medicoor unclaimed+stale (still lists deceased founder), X @SolidarityHeal1 since May 2021. Services: gen med, vaccination, surgery, lab panels, maternity, ultrasound/X-ray; reviews cite cardiologist+pharmacy; Zenithe accredited. Among Buea district top-3 most-solicited facilities (PAMJ 2023, BMRI 2025). Pitch: attach bilingual site+WA booking+same-day lab results to GBP; foundation/grant visibility; claim medicoor; 24h emergency bar. FUs M+2/M+4/M+7. [15 Sep send morning: 677 61 57 57 not registered on WhatsApp per King; voice line only, never cold-call; MITOC now leads Tue 08:35; Solidarity -&gt; admin-line check, else Wed sealed card]</t>
+          <t>Clinic lead #1, research-standard corrected 15 Sep (see sales/RESEARCH-STANDARD.md error #1). Not-for-profit CIG founded Aug 1998 by late Dr Peter Nde Fon (UB public health chair, obituary verified). GBP 4.0 stars/54 reviews/21 photos/24h, Untarred Malingo St plus code 575J+7M, NO website ('Add website'), medicoor unclaimed+stale (still lists deceased founder), X @SolidarityHeal1 since May 2021. Services: gen med, vaccination, surgery, lab panels, maternity, ultrasound/X-ray; reviews cite cardiologist+pharmacy; Zenithe accredited. Among Buea district top-3 most-solicited facilities (PAMJ 2023, BMRI 2025). Pitch: attach bilingual site+WA booking+same-day lab results to GBP; foundation/grant visibility; claim medicoor; 24h emergency bar. FUs M+2/M+4/M+7. [15 Sep send morning: 677 61 57 57 not registered on WhatsApp per King; voice line only, never cold-call; MITOC now leads Tue 08:35; Solidarity -&gt; admin-line check, else Wed sealed card] | 15 Sep PM RENAME: live concept is /clinic-bonaberi.html (LIVE, partial hand-rename by King; canonical repo build fully renamed to Douala/BMC, redeploys with amk-site.zip). Solidarity (Buea) warm-yes link uses it with placeholder caption; ask King if he wants a Buea/city-neutral variant + matching mockup-clinic image.</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5469,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>YES named: site/mitoc.html (built 15 Sep, send after warm yes)</t>
+          <t>YES named: site/mitoc.html (built 15 Sep, send after warm yes); LIVE at https://mitoc-concept.vercel.app</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">

</xml_diff>

<commit_message>
St Theresa first reply: soft-ack + 14 Oct FU logged (24h chat, verbatim saved); Douala remote sweep #1 (25 candidates, hot list, verification SOP)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -4677,9 +4677,29 @@
           <t>A</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>YES 15 Sep 15:45 WA by King (text-only msg 1, 679 15 10 75)</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>YES Tue 15 Sep 20:44 (verbatim): 'Gd evening we already have one in the making which will be ready by October. If you had gotten to me earlier then we could have used your system but it's already late.'</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>SOFT OBJECTION = competitor/in-house build in progress, ETA October. Soft-ack reply DRAFTED for King to send same evening (20:44 reply, before 21:00 window): congrats, fees+WhatsApp-admissions checklist, free second-opinion offer if it slips, permission to check back at launch. NO mockup/link pushed (would damage). 24h disappearing messages on this chat.</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>Wed 14 Oct 2026 (site promised for October — check-in: is it live? free honest review incl. WA admissions/bilingual/fees/3G); FU2 Wed 4 Nov if silent; then stop. No TikTok DM fallback (engaged on WA).</t>
+        </is>
+      </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM: msg 1 out (1 tick, not yet delivered to handset). Personal WA line (lay private = likely proprietor pocket = buyer). Mockup image went to later schools first; include image with the link on reply.</t>
+          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM: msg 1 out (1 tick, not yet delivered to handset). Personal WA line (lay private = likely proprietor pocket = buyer). Mockup image went to later schools first; include image with the link on reply. | 15 Sep 20:44 FIRST REPLY OF THE CAMPAIGN: site 'in the making, ready October, already late'. Soft-ack branch only. Watch the October launch (check Google/FB): template/student builds commonly miss WhatsApp admissions, bilingual toggle, fees pages and 3G speed = re-open wedge. Verified GCE Board 2026 marking centre (camgceb.org) — usable compliment at FU.</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="25" min="1" max="1"/>
@@ -6763,6 +6783,45 @@
       <c r="K41" t="inlineStr">
         <is>
           <t>King phone-verified: COMOBIL + SAHISCOL not on WhatsApp; declined Facebook Page + Douala trip this week. Both parked with revival triggers (COMOBIL #1 revival). Kill list now OraCare + Sasse (+NHICHS email Tue). New sourcing rule: reachable channel before high score. Tue batch 8-10 channel-qualified D/E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Sends: MITOC 08:35, Baptist ~12:00 (BOARD inbound-only), Baird 14:41 (img+text), St Theresa 15:45 (text). St Theresa replied 20:44 (site in making, October) -&gt; soft-ack, FU 14 Oct. Videos + SEO addendum produced; nationwide remote-first approved.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Addendum #3 conversion-design standard from 8-video study; proof + follow CTAs and 52px mobile tap targets in clinic/school generators (regenerated); St Theresa soft-ack delivered 22:25 (timer 90d), CRM/Daily Ops updated
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -4689,17 +4689,17 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>SOFT OBJECTION = competitor/in-house build in progress, ETA October. Soft-ack reply DRAFTED for King to send same evening (20:44 reply, before 21:00 window): congrats, fees+WhatsApp-admissions checklist, free second-opinion offer if it slips, permission to check back at launch. NO mockup/link pushed (would damage). 24h disappearing messages on this chat.</t>
+          <t>SENT by King Tue 15 Sep 22:25 (screenshot confirmed): congratulations + two launch must-haves (fees visible on phone; admissions straight into WhatsApp, EN+FR) + free honest second-opinion offer if October slips + permission to check back at launch + contact-save ask + GCE well-wish. King changed chat timer 24h -&gt; 90 days, history now retained. No mockup/link pushed. STAGE parked-warm. FU1 Wed 14 Oct 2026 (site live? free review: WA admissions, bilingual, fees, mobile, speed); FU2 Wed 4 Nov 2026 if silent; then STOP. First campaign reply (15 Sep: 4 sent, 1 reply).</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>Wed 14 Oct 2026 (site promised for October — check-in: is it live? free honest review incl. WA admissions/bilingual/fees/3G); FU2 Wed 4 Nov if silent; then stop. No TikTok DM fallback (engaged on WA).</t>
+          <t>2026-10-14 (FU1 launch check); 2026-11-04 (FU2, then stop)</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM: msg 1 out (1 tick, not yet delivered to handset). Personal WA line (lay private = likely proprietor pocket = buyer). Mockup image went to later schools first; include image with the link on reply. | 15 Sep 20:44 FIRST REPLY OF THE CAMPAIGN: site 'in the making, ready October, already late'. Soft-ack branch only. Watch the October launch (check Google/FB): template/student builds commonly miss WhatsApp admissions, bilingual toggle, fees pages and 3G speed = re-open wedge. Verified GCE Board 2026 marking centre (camgceb.org) — usable compliment at FU.</t>
+          <t>Walk-In-Batch-2026-09-15. Pain: parents find only FB/yahoo, no website. Bilingual international comprehensive. Get WA + permission, preview by 4pm. | INVITATION-FIRST 14 Sep: TikTok @stibccol ACTIVE (Bilingualism Day/Miss St Theresa posts 14 Sep 2026) = DM channel like Sasse; official FB page lists 679 15 10 75 (verify WA profile tonight). YouTube 2022 "for more info" 677 36 19 11 likely media person, do not pitch. [OWNER-BUYER confirmed type: lay private 15 Sep; remains in active plan] | 15 Sep PM: msg 1 out (1 tick, not yet delivered to handset). Personal WA line (lay private = likely proprietor pocket = buyer). Mockup image went to later schools first; include image with the link on reply. | 15 Sep 20:44 FIRST REPLY OF THE CAMPAIGN: site 'in the making, ready October, already late'. Soft-ack branch only. Watch the October launch (check Google/FB): template/student builds commonly miss WhatsApp admissions, bilingual toggle, fees pages and 3G speed = re-open wedge. Verified GCE Board 2026 marking centre (camgceb.org) — usable compliment at FU. | Soft-ack delivered 22:25; chat timer now 90 days (was 24h).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
St Theresa reply #2 (22:51): follow-up explicitly invited — stage parked-warm-with-permission, FU 14 Oct now welcomed; CRM + Daily Ops updated
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads/leads_50.xlsx
+++ b/leads/leads_50.xlsx
@@ -1163,10 +1163,10 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="B29:E29"/>
@@ -4684,12 +4684,12 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>YES Tue 15 Sep 20:44 (verbatim): 'Gd evening we already have one in the making which will be ready by October. If you had gotten to me earlier then we could have used your system but it's already late.'</t>
+          <t>YES Tue 15 Sep 20:44 (verbatim): 'Gd evening we already have one in the making which will be ready by October. If you had gotten to me earlier then we could have used your system but it's already late.' | REPLY #2 Tue 22:51 (verbatim): 'Ok thanks you can get back to me for a follow up' = EXPLICIT permission for the October check-in.</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>SENT by King Tue 15 Sep 22:25 (screenshot confirmed): congratulations + two launch must-haves (fees visible on phone; admissions straight into WhatsApp, EN+FR) + free honest second-opinion offer if October slips + permission to check back at launch + contact-save ask + GCE well-wish. King changed chat timer 24h -&gt; 90 days, history now retained. No mockup/link pushed. STAGE parked-warm. FU1 Wed 14 Oct 2026 (site live? free review: WA admissions, bilingual, fees, mobile, speed); FU2 Wed 4 Nov 2026 if silent; then STOP. First campaign reply (15 Sep: 4 sent, 1 reply).</t>
+          <t>STAGE parked-warm-with-permission (upgraded after reply #2 22:51: they invited the follow-up). SENT by King Tue 15 Sep 22:25 (screenshot confirmed): congratulations + two launch must-haves (fees visible on phone; admissions straight into WhatsApp, EN+FR) + free honest second-opinion offer if October slips + permission to check back at launch + contact-save ask + GCE well-wish. King changed chat timer 24h -&gt; 90 days, history now retained. No mockup/link pushed. STAGE parked-warm. FU1 Wed 14 Oct 2026 (site live? free review: WA admissions, bilingual, fees, mobile, speed); FU2 Wed 4 Nov 2026 if silent; then STOP. First campaign reply (15 Sep: 4 sent, 1 reply). King to send short same-night close (confirm October, contact-save, GCE well-wish). FU1 Wed 14 Oct 2026: is the site live? free honest review (WA admissions one tap, EN+FR fees visible, mobile, speed) — arrive as the invited check-in, not a chase; FU2 Wed 4 Nov if silent; then STOP. 90-day chat timer retains full history.</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">

</xml_diff>